<commit_message>
Final revisions to analysis
</commit_message>
<xml_diff>
--- a/Output/EK_model_results.xlsx
+++ b/Output/EK_model_results.xlsx
@@ -14,8 +14,7 @@
     <sheet name="part4_real_wage_expenditure" sheetId="5" state="visible" r:id="rId5"/>
     <sheet name="part4_regressions" sheetId="6" state="visible" r:id="rId6"/>
     <sheet name="part5_comparison" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet name="part5_regressions" sheetId="8" state="visible" r:id="rId8"/>
-    <sheet name="settings_and_checks" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet name="settings_and_checks" sheetId="8" state="visible" r:id="rId8"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -10737,7 +10736,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G7"/>
+  <dimension ref="A1:H7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -10753,25 +10752,30 @@
       </c>
       <c r="C1" t="inlineStr">
         <is>
+          <t>intercept</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
           <t>slope</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="E1" t="inlineStr">
         <is>
           <t>std_err</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="F1" t="inlineStr">
         <is>
           <t>t_stat</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="G1" t="inlineStr">
         <is>
           <t>R2</t>
         </is>
       </c>
-      <c r="G1" t="inlineStr">
+      <c r="H1" t="inlineStr">
         <is>
           <t>N</t>
         </is>
@@ -10789,18 +10793,21 @@
         </is>
       </c>
       <c r="C2" t="n">
+        <v>0</v>
+      </c>
+      <c r="D2" t="n">
         <v>-0.25</v>
       </c>
-      <c r="D2" t="n">
+      <c r="E2" t="n">
         <v>0</v>
       </c>
-      <c r="E2" t="n">
+      <c r="F2" t="n">
         <v>-2560207327372.133</v>
       </c>
-      <c r="F2" t="n">
+      <c r="G2" t="n">
         <v>1</v>
       </c>
-      <c r="G2" t="n">
+      <c r="H2" t="n">
         <v>40</v>
       </c>
     </row>
@@ -10816,18 +10823,21 @@
         </is>
       </c>
       <c r="C3" t="n">
-        <v>-0.078165</v>
+        <v>7.9239e-06</v>
       </c>
       <c r="D3" t="n">
-        <v>0.012986</v>
+        <v>-0.07816451369999999</v>
       </c>
       <c r="E3" t="n">
-        <v>-6.019167</v>
+        <v>0.0129859364</v>
       </c>
       <c r="F3" t="n">
-        <v>0.48808</v>
+        <v>-6.0191665313</v>
       </c>
       <c r="G3" t="n">
+        <v>0.4880801189</v>
+      </c>
+      <c r="H3" t="n">
         <v>40</v>
       </c>
     </row>
@@ -10843,18 +10853,21 @@
         </is>
       </c>
       <c r="C4" t="n">
-        <v>0.00366</v>
+        <v>-1.82473e-05</v>
       </c>
       <c r="D4" t="n">
-        <v>0.000357</v>
+        <v>0.003659954</v>
       </c>
       <c r="E4" t="n">
-        <v>10.246552</v>
+        <v>0.0003571888</v>
       </c>
       <c r="F4" t="n">
-        <v>0.734251</v>
+        <v>10.2465524087</v>
       </c>
       <c r="G4" t="n">
+        <v>0.7342505629</v>
+      </c>
+      <c r="H4" t="n">
         <v>40</v>
       </c>
     </row>
@@ -10870,18 +10883,21 @@
         </is>
       </c>
       <c r="C5" t="n">
-        <v>-0.285646</v>
+        <v>-1.7639e-06</v>
       </c>
       <c r="D5" t="n">
-        <v>0.006</v>
+        <v>-0.2856455534</v>
       </c>
       <c r="E5" t="n">
-        <v>-47.606433</v>
+        <v>0.0060001462</v>
       </c>
       <c r="F5" t="n">
-        <v>0.98351</v>
+        <v>-47.6064325089</v>
       </c>
       <c r="G5" t="n">
+        <v>0.9835096099</v>
+      </c>
+      <c r="H5" t="n">
         <v>40</v>
       </c>
     </row>
@@ -10897,18 +10913,21 @@
         </is>
       </c>
       <c r="C6" t="n">
-        <v>-0.093427</v>
+        <v>5.9456e-06</v>
       </c>
       <c r="D6" t="n">
-        <v>0.014407</v>
+        <v>-0.09342706570000001</v>
       </c>
       <c r="E6" t="n">
-        <v>-6.484854</v>
+        <v>0.0144069663</v>
       </c>
       <c r="F6" t="n">
-        <v>0.525316</v>
+        <v>-6.4848535053</v>
       </c>
       <c r="G6" t="n">
+        <v>0.5253164062</v>
+      </c>
+      <c r="H6" t="n">
         <v>40</v>
       </c>
     </row>
@@ -10924,18 +10943,21 @@
         </is>
       </c>
       <c r="C7" t="n">
-        <v>0.003974</v>
+        <v>-1.96739e-05</v>
       </c>
       <c r="D7" t="n">
-        <v>0.000471</v>
+        <v>0.0039736989</v>
       </c>
       <c r="E7" t="n">
-        <v>8.438827</v>
+        <v>0.0004708828</v>
       </c>
       <c r="F7" t="n">
-        <v>0.6520590000000001</v>
+        <v>8.4388270461</v>
       </c>
       <c r="G7" t="n">
+        <v>0.6520586287</v>
+      </c>
+      <c r="H7" t="n">
         <v>40</v>
       </c>
     </row>
@@ -12282,85 +12304,6 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E3"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <sheetData>
-    <row r="1">
-      <c r="A1" t="inlineStr">
-        <is>
-          <t>outcome</t>
-        </is>
-      </c>
-      <c r="B1" t="inlineStr">
-        <is>
-          <t>slope on (1 - y0)</t>
-        </is>
-      </c>
-      <c r="C1" t="inlineStr">
-        <is>
-          <t>std_err</t>
-        </is>
-      </c>
-      <c r="D1" t="inlineStr">
-        <is>
-          <t>R2</t>
-        </is>
-      </c>
-      <c r="E1" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>real wage difference (pp)</t>
-        </is>
-      </c>
-      <c r="B2" t="n">
-        <v>0.195304</v>
-      </c>
-      <c r="C2" t="n">
-        <v>0.007131</v>
-      </c>
-      <c r="D2" t="n">
-        <v>0.951781</v>
-      </c>
-      <c r="E2" t="n">
-        <v>40</v>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>real expenditure difference (pp)</t>
-        </is>
-      </c>
-      <c r="B3" t="n">
-        <v>2.365849</v>
-      </c>
-      <c r="C3" t="n">
-        <v>0.007677</v>
-      </c>
-      <c r="D3" t="n">
-        <v>0.9996</v>
-      </c>
-      <c r="E3" t="n">
-        <v>40</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
   <dimension ref="A1:B11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>

</xml_diff>